<commit_message>
Daily EOD data and reports for 2026-09-24
</commit_message>
<xml_diff>
--- a/asx_eod_output/Report_XLSX/Report_20260924.xlsx
+++ b/asx_eod_output/Report_XLSX/Report_20260924.xlsx
@@ -488,24 +488,24 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>1.89</v>
+        <v>1.895</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>-0.105</v>
+        <v>-0.1</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>-5.26%</t>
+          <t>-5.01%</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
         <v>153181</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>289512.09</v>
+        <v>290277.99</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>-16084.01</v>
+        <v>-15318.1</v>
       </c>
     </row>
     <row r="5">
@@ -542,24 +542,24 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>60.95</v>
+        <v>61.02</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>-1.12</v>
+        <v>-1.05</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>-1.80%</t>
+          <t>-1.69%</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
         <v>8000</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>487600</v>
+        <v>488160</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>-8960</v>
+        <v>-8400</v>
       </c>
     </row>
     <row r="7">
@@ -596,14 +596,14 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>149.48</v>
+        <v>149.98</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>-1.57</v>
+        <v>-1.07</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>-1.04%</t>
+          <t>-0.71%</t>
         </is>
       </c>
       <c r="E8" s="3" t="n">
@@ -623,24 +623,24 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>0.92</v>
+        <v>0.925</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>-0.025</v>
+        <v>-0.02</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-2.65%</t>
+          <t>-2.12%</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
         <v>10000</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>9200</v>
+        <v>9250</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>-250</v>
+        <v>-200</v>
       </c>
     </row>
     <row r="10">
@@ -650,24 +650,24 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>179.415</v>
+        <v>179.12</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.175</v>
+        <v>-0.12</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.10%</t>
+          <t>-0.07%</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
         <v>4000</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>717660</v>
+        <v>716480</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>700</v>
+        <v>-480</v>
       </c>
     </row>
     <row r="11">
@@ -677,24 +677,24 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>0.22</v>
+        <v>0.23</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>-0.015</v>
+        <v>-0.005</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>-6.38%</t>
+          <t>-2.13%</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
         <v>20000</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>4400</v>
+        <v>4600</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>-300</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="12">
@@ -704,24 +704,24 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>16.19</v>
+        <v>16.25</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>-0.43</v>
+        <v>-0.37</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>-2.59%</t>
+          <t>-2.23%</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
         <v>3045</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>49298.55</v>
+        <v>49481.25</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>-1309.35</v>
+        <v>-1126.65</v>
       </c>
     </row>
     <row r="13">
@@ -758,24 +758,24 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>0.093</v>
+        <v>0.094</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>-0.002</v>
+        <v>-0.001</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>-2.11%</t>
+          <t>-1.05%</t>
         </is>
       </c>
       <c r="E14" s="3" t="n">
         <v>9412</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>875.3200000000001</v>
+        <v>884.73</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>-18.82</v>
+        <v>-9.41</v>
       </c>
     </row>
     <row r="15">
@@ -812,14 +812,14 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>34.145</v>
+        <v>34.13</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>-0.615</v>
+        <v>-0.63</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>-1.77%</t>
+          <t>-1.81%</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
@@ -839,24 +839,24 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>31.595</v>
+        <v>31.61</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.465</v>
+        <v>0.48</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>1.49%</t>
+          <t>1.54%</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
         <v>1288</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>40694.36</v>
+        <v>40713.68</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>598.92</v>
+        <v>618.24</v>
       </c>
     </row>
     <row r="18">
@@ -870,10 +870,10 @@
       <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="7" t="inlineStr"/>
       <c r="F18" s="8" t="n">
-        <v>1786192.68</v>
+        <v>1786800.01</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>-24235.26</v>
+        <v>-23627.92</v>
       </c>
     </row>
   </sheetData>

</xml_diff>